<commit_message>
Updates to styles for rates
</commit_message>
<xml_diff>
--- a/documentation/Automated Testing Pulse.xlsx
+++ b/documentation/Automated Testing Pulse.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hughw\OneDrive\Documents\ennovative\ProjectsNewLaptop\CFSuiteFullBuildUnpackaged\CFSuiteCumulusFullBuildUnpackaged\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bfadeac5487ed7d8/Documents/ennovative/ProjectsNewLaptop/CFSuiteFullBuildUnpackaged/CFSuiteCumulusFullBuildUnpackaged/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3089D2BE-D956-4F10-81B0-18446B1956C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{3089D2BE-D956-4F10-81B0-18446B1956C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC2E4E3D-AC1E-41E5-A2B5-D9D1088948FB}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="885" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Automated Tests" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="71">
   <si>
     <t>TEST SCRIPTS</t>
   </si>
@@ -71,13 +72,875 @@
   </si>
   <si>
     <t>Decision Maker</t>
+  </si>
+  <si>
+    <t>1.From app launcher open CFSuite Pulse​
+2.Select the Surveys Tab​
+3.Select [New]​
+4.Enter a survey name: ‘Case Closed – {category name}’​
+5.Develop the survey​
+.Background image / branding​
+.Edit or hide the welcome screen message​
+.Add questions and pages (Net promoter type for ranking) ​
+.Edit or hide the thankyou message​
+6.Click ‘Activate’ and close the Builder​​
+7.Save​</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">1.Open the Survey Record from the Survey Tab ​
+2.Locate the question you want to set Callback. ​
+3.select the value that you want to trigger the callback. 
+4.select the category journey of the case you want to create. 
+5.In the case below there is a question "Would you like a callback?" 
+6.Select “YES” on the radio group field. 
+7.Add the category journey record (the case will be created of the CJ record you selected)
+8.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">When a survey is answered now and the user asks for a callback, a case will be created as a child of the original case.   </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1. Go to a Contact that has a value 'Email' on the field 'Preferred Notification (Customer Survey)'
+2. Create a sample case from that Contact
+(i.e) Trees, Parks and Public Spaces -&gt; Maintenance Schedule -&gt; Tree Maintenance
+3. Once the case is created, Mark the case as '</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Closed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">'
+Status -&gt; Closed
+Reason -&gt; Work Complete
+4. An email with the Survey link will be sent to the Contact's Email ID.
+From </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>City Of Whittlesea &lt;council@whittlesea.vic.gov.au&gt;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1. Go to a Contact that has a value 'Email' on the field 'Preferred Notification (Customer Survey)'
+2. Create a sample case from that Contact
+(i.e) Trees, Parks and Public Spaces -&gt; Maintenance Schedule -&gt; Tree Maintenance
+3. Once the case is created, Mark the case as '</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Closed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">'
+Status -&gt; Closed
+Reason -&gt; Work Complete
+4. An email with the Survey link will be sent to the Contact's Email ID.
+From </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">City Of Whittlesea &lt;council@whittlesea.vic.gov.au&gt;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">5. Click on the survey link. It will open the survey in a new browser window
+6. Answer the questions one by one. On Page 2 of the Survey, provide feedback as below for these questions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>My request was resolved promptly and efficiently</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Below 3 Stars
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>How many times did you need to contact us to resolve your enquiry?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">My request is not resolved
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Would you like us to contact you?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Yes
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>7. And then continue to submit the survey
+8. Now in CFsuite console, go to Customer Satisfaction Survey -&gt; All cases. You can see a new case is created with a Request reason as '</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Close the loop</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>'.
+9. And it has a Parent case linked to it. The Parent case number will be the Case that was closed above.
+10. Go to the Parent Case. And you can view the Survey responses from the 'Survey Invitations and Responses' component on the case record page.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1. Go to a Contact that has a value 'Email' on the field 'Preferred Notification (Customer Survey)'
+2. Create a sample case from that Contact
+(i.e) Trees, Parks and Public Spaces -&gt; Maintenance Schedule -&gt; Tree Maintenance
+3. Once the case is created, Mark the case as '</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Closed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">'
+Status -&gt; Closed
+Reason -&gt; Work Complete
+4. An email with the Survey link will be sent to the Contact's Email ID.
+From </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">City Of Whittlesea &lt;council@whittlesea.vic.gov.au&gt;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">5. Click on the survey link. It will open the survey in a new browser window
+6. Answer the questions one by one. On Page 2 of the Survey, provide feedback as below for these questions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>My request was resolved promptly and efficiently</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Below 3 Stars
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>How many times did you need to contact us to resolve your enquiry?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">My request is not resolved
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Would you like us to contact you?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">No
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>7. And then continue to submit the survey
+8. Now in CFSuite console, go to Customer Satisfaction Survey -&gt; All cases. There will be no new cases created.</t>
+    </r>
+  </si>
+  <si>
+    <t>​1.​From app launcher open CFSuite Pulse​
+2.Select campaigns ​
+3.Click on [Create CFSuite Pulse Campaign] in top right corner​
+4.Enter a campaign name 
+5.Select the Survey from the dropdown​
+6.Select ‘Campaign Survey Email’ from the dropdown list​
+7.Select ‘Campaign Survey SMS’ from the dropdown list​
+8.Add a short description such as ‘Training campaign for Pulse 360’​
+9.Select ‘No’ to activating the campaign now​
+10.Click [Next]
+11.This creates your campaign record.
+​
+​</t>
+  </si>
+  <si>
+    <t>1.Open the campaign record
+2.From the related list of campaign members 
+3.Add Leads manually​
+4.Clicking [Add lead] button then searching by name​
+(very time consuming and not very easy, plus the contacts list is not useful or complete)​
+5.When all added click [Next]​
+6.Click [Submit]​
+7.Contacts will be added to the campaign as members​
+Add contacts from a CSV Upload​
+8.Click on “Import Leads and Contacts" button​
+9.Data import wizard opens up​, click on Leads
+10.Select ​Add new &amp; Update existing records then set your field matching criteria
+11.Upload your Contact CSV file, then click Next
+12.Your file will be automapped to the existing salesforce fields, then click next
+12.Leave status as ‘pending’ and ‘keep member status’​
+13.Click [Submit] – which will add members and email once done
+14.The members will be added from the csv file upload​
+15.Any duplicate email addresses will only be added once</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From within the campaign you created and added campaign members:
+1.Navigate to the "Launch Campaign" widget on the right side of the campaign page.
+2.Click the Preview button.
+3.The system will open a "Launch Campaign Preview" window displaying a list view of the campaign members.
+4.In the list view, locate the Preferred Contact column, which shows each campaign member's preferred notification method for customer surveys.
+5.Confirm that each campaign member has either SMS or Email specified as their preferred contact method.
+</t>
+  </si>
+  <si>
+    <t>From within the campaign you created​
+1.Click on the Details tab​
+2.Set the following​
+.[Active] to TRUE​
+.[Status] from ‘Planned’ to ‘In Progress’​
+3.The Launch Campaign control displays the number fo Emails and SMS that will be sent​
+4.To launch click [Send]​
+5.The system will trigger bulk SMS and email delivery to all recipients​
+6.Respond to the survey and refresh the survey record – status of members updates to ‘responded’​
+​</t>
+  </si>
+  <si>
+    <t>1.From the App Launcher, open Leads.
+2.Select the list view ‘All Open Leads’.
+Expected Results:
+3.Users with the CFSuite Pulse Admin permission set can only view and access all lead records.
+4.Users without the CFSuite Pulse Admin permission set cannot view or access any lead records.</t>
+  </si>
+  <si>
+    <t>1.Login as Pulse user
+2. From app launcher open CFSuite Pulse​
+3. I should be able to see a CSAT Dashboard with below Reports
+CSAT Trend
+Post Service Delivery CSAT Composition
+Leaderboard
+Drivers
+Verbatim Responses</t>
+  </si>
+  <si>
+    <t>1.From App Launcher, go to Contacts.
+2.Switch to a list view that shows Contacts (e.g., Individual contacts).
+3.Select one or more contact records using the checkboxes.
+4.Click Add Contacts to Campaign at the top of the list view.
+5.In the pop-up, select the Campaign and choose a Member Status.
+6.Click Submit.
+7.Verify the selected contacts are now added as Campaign Members.
+Use the Add to Campaign Button (Reports)
+1.From App Launcher, open Reports.
+2.Open a Contact or Account report e.g "New Accounts &amp; Contact report"
+3.In the top-right toolbar, click the dropdown arrow (Actions).
+4.Click Add to Campaign.
+5.Choose the Campaign and Member Status.
+6.Click Submit.
+7.Verify the selected records appear as Campaign Members on the campaign.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">1.Go to the Campaign record in Salesforce.
+2.Click the Related tab, then click CFSuite Campaign Actions.
+3.Click New to create a new campaign action.
+4.Enter a value in the CFSuite Campaign Action Name field.
+5.In the Action Type field, select Reminder.
+6.In the Days from Invite field, specify the number of days after the original invite when the reminder should be sent.
+7.(Optional) In the Reminder Day field, specify the day of the week the reminder should be sent.
+8.In the Email Template field, select the email template to be used for the reminder.
+9.In the SMS Template field, select the SMS template to be used for the reminder.
+10.Click Save to create the reminder action.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Please note :
+If email &amp; SMS intergration is </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NOT</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> done in your test environment; the Campaign reminders SMS or Emails will </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NOT</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> be sent through to the Campaign Member(s), therefore you</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> MUST</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> check that:-
+a)System Populates the survey invitation record with the campaign message
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> if SMS &amp; email intergration is </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DONE</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: A campaign reminder is created and scheduled to send the selected email or SMS template after the defined number of days or on the specified day after the campaign invite is sent. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>1.Log in to the community portal 
+2.Click "Make Request" tile 
+3.Select Pets, Animals, Pests &gt; Cat &amp; Dog registration &gt; Request a replacement tag
+4.Select request location etc then submit request
+5.At the end of case creation page a quick poll question comes up ."How did we do today?"
+6. Click any of the stars to complete the quick poll
+7.A survey hyperlink "Provide detailed feedback on your experience" appears
+8.Upon clicking the hyperlink ,user gets redirected to a new browser window with survey questions.
+9. Complete the survey questions .
+10. Confirm that Customer Insight is record is created</t>
+  </si>
+  <si>
+    <t>1.Go to a scheduled Campaign record.
+2. Navigate to the Cancel Campaign send widget on the right hand side.
+3.Click the Cancel Campaign schedule button.
+4.This will cancel the the scheduled jobs from sending the campaign 
+5.The scheduled status gets updated from "Scheduled" to "Not scheduled"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Go to a Campaign Record
+2.Ensure the campaign record has Campaign members added 
+3.Navigate to the Campasign schedule section then update the Campaign send date &amp; time fields.
+4.Save the changes then navigate to the top right side of the campaign page
+5.Once you are happy with the campaign, click the Send button as you would for any normal campaign. 
+6.You will see a confirmation message, and the campaign status will update to scheduled. 
+If you click send on a scheduled campaign its supposed to run the campaign  according the send date/time field </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.An email with unsubscribe hyperlink is delievered to recipients email.
+2.Upon clicking the unsubscribe hyperlink, they get redirected to a new unsubscribe browser winddow.
+3.The users email address gets automatically populated in the "Confirm your email" field.
+4.Upon confirming that the email address is accurate, the user can click the unsubscribe button.
+This should trigger the unsubscribe function to update the user's record;
+5.The user's contact record gets updated .The Preferred Notification (Customer Survey) field will have the value "Opt out Surveys".
+</t>
+  </si>
+  <si>
+    <t>1. A Survey should be created and Activated
+2. Above created Survey should be available in Survey tab on CFSuite Pulse App
+3.Pulse Users without the permission sets will not have a button to create New surveys.</t>
+  </si>
+  <si>
+    <t>Verify that the user can:
+1.add a Single Response question that triggers the case creation. 
+2.select a Category Journey for the callback case.</t>
+  </si>
+  <si>
+    <t>1. A case should be created and Closed
+2. A survey email should be sent to Customer's email</t>
+  </si>
+  <si>
+    <t>1. A case should be created and Closed
+2. A survey email should be sent to Customer's email
+3. A child case - 'Close the loop survey' cases should be created and assigned to 'Customer Satisfaction Survey' Queue</t>
+  </si>
+  <si>
+    <t>1. A case should be created and Closed
+2. A survey email should be sent to Customer's email
+3. A child case - 'Close the loop survey' cases should not be created</t>
+  </si>
+  <si>
+    <t>1. A Campaign should be created
+2. Above created Campaign should be available in Campaign tab on CFSuite Pulse App.
+3.Pulse users without the pulse permission sets assigned to them can't create campaigns.</t>
+  </si>
+  <si>
+    <t>1. Leads added manually and through CSV as campaign members
+2.Pulse users without the permission sets can't add or upload Leads to a campaign
+3. If the CSV file is loaded without proper Lead Field names, the Data Import wizard should throw error on Field mapping step / druing the file upload.</t>
+  </si>
+  <si>
+    <t>1. Preview from launch Campaign component should list the loaded leads with Pref comms
+2.The Launch Campaign Preview window will display values from Prefered Notification(survey) field.</t>
+  </si>
+  <si>
+    <t>1.The bulk emails should be sent from Campaigns to the loaded campaign members.
+2.Campaign members with Preferred Notification (surveys) set as Opt out of surveys should not recieve the campaign email.
+3..Campaign members with Preferred Notification (surveys) set as email should recieve the campaign email.</t>
+  </si>
+  <si>
+    <t>1.Loaded Lead Records should Only be accessed by the CFSuite Pulse Admin, with pulse permission set.
+2.Only the records that the user has access to should be visible on the listviews.</t>
+  </si>
+  <si>
+    <t>The CSAT Dashboard should be available on the Home page of CFSuite Pulse app to CFSuite admin users with permission set assigned .
+These Dashboard reports should be visible on Homepage
+1.CSAT Trend
+2.Post Service Delivery CSAT Composition
+3.Leaderboard
+4.Drivers
+5.Verbatim Responses</t>
+  </si>
+  <si>
+    <t>User can select one or more contacts from a list view to add as Campaign member.
+- Add Contacts to Campaign button from the list view is visible
+- User can add contacts from a report to Campaign as campaign members
+- selected records are added as Campaign Members and visible on the campaign record.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Please confirm that:
+1.Users can to configure reminder actions in CFSuite Campaign Actions on the campaign
+2.Reminders send only when the customer has not opted out of surveys.
+3.Reminders send only when the member has not responded to the survey.
+Incase you perform  campaign reminders test on an org before sms &amp; email integration, please check that the system can:
+1.Populate the survey invitation record with the campaign message
+</t>
+  </si>
+  <si>
+    <t>1. Users can provide a star rating on the Thank You page.
+2.When a star rating is given, users have the option to provide additional written feedback below the rating.
+3.Submission of the star rating and feedback automatically creates a Customer Insight record.
+4.If the user clicks the link provided on the Thank You page, a new survey is generated (the survey does not include a star rating question).
+5.When the survey is completed, it is linked to the original Customer Insight record for reference and tracking.</t>
+  </si>
+  <si>
+    <t>1.Cancel Campaign schedule is visible to users
+2.When a user cancels a scheduled campaign the status gets updated from "Scheduled" to "Not scheduled"</t>
+  </si>
+  <si>
+    <t>1.The campaign’s Status updates from “Not Scheduled” to “Scheduled.”
+2.A scheduled job is created to run the campaign at the specified Send Date/Time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.The unsubscribe function is inbuilt in an email template.
+2.Clicking the unsubscribe hyperlink redirects to a new browser window.
+3.Customer's email address automaticlly gets populated on the email field and is non-editable.
+4. Clicking the unsubscribe button triggers a fuction that updates the contact record's Preferred Notification (Customer Survey) field to "Opt Out of surveys"
+5.There is a confirmation screen comes up  after user unsubscribing.
+</t>
+  </si>
+  <si>
+    <t>Create New Survey as a Pulse user</t>
+  </si>
+  <si>
+    <t>Enable Case Categories for Survey as an Admin</t>
+  </si>
+  <si>
+    <t>Send Survey Email on case Closure</t>
+  </si>
+  <si>
+    <t>Create a Follow up case from Survey</t>
+  </si>
+  <si>
+    <t>Skip the 'Close the loop case' from Survey</t>
+  </si>
+  <si>
+    <t>Create Campaign</t>
+  </si>
+  <si>
+    <t>Import Leads into campaign as Campaign Members</t>
+  </si>
+  <si>
+    <t>Preview &amp; set Preferred method of comms for leads</t>
+  </si>
+  <si>
+    <t>Campaign – activate and send​</t>
+  </si>
+  <si>
+    <t>Security on leads records.</t>
+  </si>
+  <si>
+    <t>Reports and Dashboards</t>
+  </si>
+  <si>
+    <t>Add Campaign members from reports or Listviews</t>
+  </si>
+  <si>
+    <t>Campaign Reminders</t>
+  </si>
+  <si>
+    <t>Community Portal Thank you page quick poll</t>
+  </si>
+  <si>
+    <t>Campaign Rescheduling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campaign Scheduling </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unsubscribe from Surveys </t>
+  </si>
+  <si>
+    <t>The Case Closure Campaign must exist first and match the name of the Case Closure Campaign setting in the CFSuite Pulse custom settings.</t>
+  </si>
+  <si>
+    <t>1.  navigate to the Unsubscribe page and unsubscribe with a non existent token.
+2.  Misc record created with Exception = Token unsubscribe — outcome: Silent-Fail-Expired</t>
+  </si>
+  <si>
+    <t>CFSuiteSettings__c custom settings need to have the fully qualified name od the Outreach preference and the Survey Preference fields.
+Survey_Comms_Preference__c: cfsuite2__Preferred_Notification_Customer_Survey__c
+Outreach_Comms_Preference__c: cfsuite2__Preferred_Notification_Outreach__c</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -124,8 +987,44 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -186,6 +1085,12 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="12">
     <border>
@@ -331,10 +1236,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -434,12 +1340,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -461,8 +1361,39 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -747,48 +1678,49 @@
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="4" width="45" customWidth="1"/>
-    <col min="5" max="7" width="55" customWidth="1"/>
+    <col min="5" max="5" width="73.85546875" customWidth="1"/>
+    <col min="6" max="7" width="55" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="43"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="41"/>
       <c r="G1" s="32"/>
-      <c r="H1" s="44" t="s">
+      <c r="H1" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
-      <c r="N1" s="40"/>
-      <c r="O1" s="40"/>
-      <c r="P1" s="40"/>
-      <c r="Q1" s="40"/>
-      <c r="R1" s="40"/>
-      <c r="S1" s="40"/>
-      <c r="T1" s="45"/>
-      <c r="U1" s="39" t="s">
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
+      <c r="K1" s="38"/>
+      <c r="L1" s="38"/>
+      <c r="M1" s="38"/>
+      <c r="N1" s="38"/>
+      <c r="O1" s="38"/>
+      <c r="P1" s="38"/>
+      <c r="Q1" s="38"/>
+      <c r="R1" s="38"/>
+      <c r="S1" s="38"/>
+      <c r="T1" s="43"/>
+      <c r="U1" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="V1" s="40"/>
-      <c r="W1" s="40"/>
-      <c r="X1" s="40"/>
-      <c r="Y1" s="40"/>
-      <c r="Z1" s="40"/>
-      <c r="AA1" s="40"/>
-      <c r="AB1" s="40"/>
-      <c r="AC1" s="40"/>
-      <c r="AD1" s="40"/>
-      <c r="AE1" s="40"/>
-      <c r="AF1" s="40"/>
+      <c r="V1" s="38"/>
+      <c r="W1" s="38"/>
+      <c r="X1" s="38"/>
+      <c r="Y1" s="38"/>
+      <c r="Z1" s="38"/>
+      <c r="AA1" s="38"/>
+      <c r="AB1" s="38"/>
+      <c r="AC1" s="38"/>
+      <c r="AD1" s="38"/>
+      <c r="AE1" s="38"/>
+      <c r="AF1" s="38"/>
     </row>
     <row r="2" spans="1:32" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
@@ -798,35 +1730,35 @@
       <c r="E2" s="1"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="44" t="s">
+      <c r="H2" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="40"/>
-      <c r="L2" s="40"/>
-      <c r="M2" s="40"/>
-      <c r="N2" s="40"/>
-      <c r="O2" s="40"/>
-      <c r="P2" s="40"/>
-      <c r="Q2" s="40"/>
-      <c r="R2" s="40"/>
-      <c r="S2" s="40"/>
-      <c r="T2" s="45"/>
-      <c r="U2" s="39" t="s">
+      <c r="I2" s="38"/>
+      <c r="J2" s="38"/>
+      <c r="K2" s="38"/>
+      <c r="L2" s="38"/>
+      <c r="M2" s="38"/>
+      <c r="N2" s="38"/>
+      <c r="O2" s="38"/>
+      <c r="P2" s="38"/>
+      <c r="Q2" s="38"/>
+      <c r="R2" s="38"/>
+      <c r="S2" s="38"/>
+      <c r="T2" s="43"/>
+      <c r="U2" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="V2" s="40"/>
-      <c r="W2" s="40"/>
-      <c r="X2" s="40"/>
-      <c r="Y2" s="40"/>
-      <c r="Z2" s="40"/>
-      <c r="AA2" s="40"/>
-      <c r="AB2" s="40"/>
-      <c r="AC2" s="40"/>
-      <c r="AD2" s="40"/>
-      <c r="AE2" s="40"/>
-      <c r="AF2" s="40"/>
+      <c r="V2" s="38"/>
+      <c r="W2" s="38"/>
+      <c r="X2" s="38"/>
+      <c r="Y2" s="38"/>
+      <c r="Z2" s="38"/>
+      <c r="AA2" s="38"/>
+      <c r="AB2" s="38"/>
+      <c r="AC2" s="38"/>
+      <c r="AD2" s="38"/>
+      <c r="AE2" s="38"/>
+      <c r="AF2" s="38"/>
     </row>
     <row r="3" spans="1:32" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -926,14 +1858,22 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:32" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:32" ht="111.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="33"/>
       <c r="B4" s="34"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="37"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="37"/>
+      <c r="C4" s="50" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" s="48" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="35"/>
+      <c r="G4" s="48" t="s">
+        <v>34</v>
+      </c>
       <c r="H4" s="14"/>
       <c r="I4" s="15"/>
       <c r="J4" s="16"/>
@@ -961,436 +1901,570 @@
       <c r="AF4" s="25"/>
     </row>
     <row r="5" spans="1:32" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="38"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="38"/>
-      <c r="G5" s="38"/>
+      <c r="A5" s="36"/>
+      <c r="B5" s="36"/>
+      <c r="C5" s="50" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="48" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="36"/>
+      <c r="G5" s="48" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="6" spans="1:32" ht="105" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="38"/>
-      <c r="B6" s="38"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="38"/>
+      <c r="A6" s="36"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="50" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" s="46" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="36" t="s">
+        <v>68</v>
+      </c>
+      <c r="G6" s="46" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="7" spans="1:32" ht="315" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="38"/>
-      <c r="B7" s="38"/>
-      <c r="C7" s="38"/>
-      <c r="D7" s="38"/>
-      <c r="E7" s="38"/>
-      <c r="F7" s="38"/>
-      <c r="G7" s="38"/>
+      <c r="A7" s="36"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="50" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="46" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="36"/>
+      <c r="G7" s="46" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="8" spans="1:32" ht="255" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="38"/>
-      <c r="B8" s="38"/>
-      <c r="C8" s="38"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="38"/>
-      <c r="G8" s="38"/>
+      <c r="A8" s="36"/>
+      <c r="B8" s="36"/>
+      <c r="C8" s="51" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="36"/>
+      <c r="G8" s="47" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="9" spans="1:32" ht="225" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="38"/>
-      <c r="B9" s="38"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="38"/>
+      <c r="A9" s="36"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="50" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="48" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="36"/>
+      <c r="G9" s="48" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="10" spans="1:32" ht="225" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="38"/>
-      <c r="B10" s="38"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="38"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="38"/>
-      <c r="G10" s="38"/>
+      <c r="A10" s="36"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="50" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="48" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="36"/>
+      <c r="G10" s="48" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="11" spans="1:32" ht="255" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="38"/>
-      <c r="B11" s="38"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="38"/>
-      <c r="E11" s="38"/>
-      <c r="F11" s="38"/>
-      <c r="G11" s="38"/>
+      <c r="A11" s="36"/>
+      <c r="B11" s="36"/>
+      <c r="C11" s="52" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="48" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" s="36"/>
+      <c r="G11" s="48" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="12" spans="1:32" ht="165" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="38"/>
-      <c r="B12" s="38"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="38"/>
-      <c r="G12" s="38"/>
+      <c r="A12" s="36"/>
+      <c r="B12" s="36"/>
+      <c r="C12" s="50" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="36"/>
+      <c r="G12" s="48" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="13" spans="1:32" ht="210" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="38"/>
-      <c r="B13" s="38"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="38"/>
-      <c r="G13" s="38"/>
+      <c r="A13" s="36"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="49" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="36"/>
+      <c r="G13" s="49" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="14" spans="1:32" ht="195" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="38"/>
-      <c r="B14" s="38"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="38"/>
-      <c r="G14" s="38"/>
+      <c r="A14" s="36"/>
+      <c r="B14" s="36"/>
+      <c r="C14" s="53" t="s">
+        <v>61</v>
+      </c>
+      <c r="D14" s="49" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" s="48" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="36"/>
+      <c r="G14" s="49" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="15" spans="1:32" ht="180" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="38"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="38"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="38"/>
-      <c r="G15" s="38"/>
+      <c r="A15" s="36"/>
+      <c r="B15" s="36"/>
+      <c r="C15" s="36" t="s">
+        <v>62</v>
+      </c>
+      <c r="D15" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" s="36"/>
+      <c r="G15" s="48" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="16" spans="1:32" ht="225" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="38"/>
-      <c r="B16" s="38"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="38"/>
-      <c r="G16" s="38"/>
+      <c r="A16" s="36"/>
+      <c r="B16" s="36"/>
+      <c r="C16" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="46" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" s="36"/>
+      <c r="G16" s="46" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="17" spans="1:7" ht="165" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="38"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="38"/>
-      <c r="G17" s="38"/>
+      <c r="A17" s="36"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="36" t="s">
+        <v>64</v>
+      </c>
+      <c r="D17" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17" s="48" t="s">
+        <v>30</v>
+      </c>
+      <c r="F17" s="36"/>
+      <c r="G17" s="48" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="18" spans="1:7" ht="195" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="38"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="38"/>
-      <c r="G18" s="38"/>
+      <c r="A18" s="36"/>
+      <c r="B18" s="36"/>
+      <c r="C18" s="36" t="s">
+        <v>65</v>
+      </c>
+      <c r="D18" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="E18" s="48" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" s="36"/>
+      <c r="G18" s="48" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="19" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="38"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="38"/>
-      <c r="G19" s="38"/>
+      <c r="A19" s="36"/>
+      <c r="B19" s="36"/>
+      <c r="C19" s="52" t="s">
+        <v>66</v>
+      </c>
+      <c r="D19" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="E19" s="48" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" s="36"/>
+      <c r="G19" s="48" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="20" spans="1:7" ht="165" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="38"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="38"/>
-      <c r="G20" s="38"/>
+      <c r="A20" s="36"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="D20" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="E20" s="48" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20" s="36"/>
+      <c r="G20" s="48" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="21" spans="1:7" ht="210" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="38"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="38"/>
+      <c r="A21" s="36"/>
+      <c r="B21" s="36"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="F21" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="G21" s="36"/>
     </row>
     <row r="22" spans="1:7" ht="345" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="38"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="38"/>
-      <c r="G22" s="38"/>
+      <c r="A22" s="36"/>
+      <c r="B22" s="36"/>
+      <c r="C22" s="36"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36"/>
     </row>
     <row r="23" spans="1:7" ht="375" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="38"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="38"/>
-      <c r="G23" s="38"/>
+      <c r="A23" s="36"/>
+      <c r="B23" s="36"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="36"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="36"/>
     </row>
     <row r="24" spans="1:7" ht="195" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="38"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="38"/>
+      <c r="A24" s="36"/>
+      <c r="B24" s="36"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="36"/>
     </row>
     <row r="25" spans="1:7" ht="150" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="38"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="38"/>
+      <c r="A25" s="36"/>
+      <c r="B25" s="36"/>
+      <c r="C25" s="36"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="36"/>
+      <c r="F25" s="36"/>
+      <c r="G25" s="36"/>
     </row>
     <row r="26" spans="1:7" ht="270" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="38"/>
-      <c r="B26" s="38"/>
-      <c r="C26" s="38"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="38"/>
-      <c r="G26" s="38"/>
+      <c r="A26" s="36"/>
+      <c r="B26" s="36"/>
+      <c r="C26" s="36"/>
+      <c r="D26" s="36"/>
+      <c r="E26" s="36"/>
+      <c r="F26" s="36"/>
+      <c r="G26" s="36"/>
     </row>
     <row r="27" spans="1:7" ht="180" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="38"/>
-      <c r="B27" s="38"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="38"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="38"/>
+      <c r="A27" s="36"/>
+      <c r="B27" s="36"/>
+      <c r="C27" s="36"/>
+      <c r="D27" s="36"/>
+      <c r="E27" s="36"/>
+      <c r="F27" s="36"/>
+      <c r="G27" s="36"/>
     </row>
     <row r="28" spans="1:7" ht="210" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="38"/>
-      <c r="B28" s="38"/>
-      <c r="C28" s="38"/>
-      <c r="D28" s="38"/>
-      <c r="E28" s="38"/>
-      <c r="F28" s="38"/>
-      <c r="G28" s="38"/>
+      <c r="A28" s="36"/>
+      <c r="B28" s="36"/>
+      <c r="C28" s="36"/>
+      <c r="D28" s="36"/>
+      <c r="E28" s="36"/>
+      <c r="F28" s="36"/>
+      <c r="G28" s="36"/>
     </row>
     <row r="29" spans="1:7" ht="360" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="38"/>
-      <c r="B29" s="38"/>
-      <c r="C29" s="38"/>
-      <c r="D29" s="38"/>
-      <c r="E29" s="38"/>
-      <c r="F29" s="38"/>
-      <c r="G29" s="38"/>
+      <c r="A29" s="36"/>
+      <c r="B29" s="36"/>
+      <c r="C29" s="36"/>
+      <c r="D29" s="36"/>
+      <c r="E29" s="36"/>
+      <c r="F29" s="36"/>
+      <c r="G29" s="36"/>
     </row>
     <row r="30" spans="1:7" ht="165" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="38"/>
-      <c r="B30" s="38"/>
-      <c r="C30" s="38"/>
-      <c r="D30" s="38"/>
-      <c r="E30" s="38"/>
-      <c r="F30" s="38"/>
-      <c r="G30" s="38"/>
+      <c r="A30" s="36"/>
+      <c r="B30" s="36"/>
+      <c r="C30" s="36"/>
+      <c r="D30" s="36"/>
+      <c r="E30" s="36"/>
+      <c r="F30" s="36"/>
+      <c r="G30" s="36"/>
     </row>
     <row r="31" spans="1:7" ht="225" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="38"/>
-      <c r="B31" s="38"/>
-      <c r="C31" s="38"/>
-      <c r="D31" s="38"/>
-      <c r="E31" s="38"/>
-      <c r="F31" s="38"/>
-      <c r="G31" s="38"/>
+      <c r="A31" s="36"/>
+      <c r="B31" s="36"/>
+      <c r="C31" s="36"/>
+      <c r="D31" s="36"/>
+      <c r="E31" s="36"/>
+      <c r="F31" s="36"/>
+      <c r="G31" s="36"/>
     </row>
     <row r="32" spans="1:7" ht="225" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="38"/>
-      <c r="B32" s="38"/>
-      <c r="C32" s="38"/>
-      <c r="D32" s="38"/>
-      <c r="E32" s="38"/>
-      <c r="F32" s="38"/>
-      <c r="G32" s="38"/>
+      <c r="A32" s="36"/>
+      <c r="B32" s="36"/>
+      <c r="C32" s="36"/>
+      <c r="D32" s="36"/>
+      <c r="E32" s="36"/>
+      <c r="F32" s="36"/>
+      <c r="G32" s="36"/>
     </row>
     <row r="33" spans="1:7" ht="210" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="38"/>
-      <c r="B33" s="38"/>
-      <c r="C33" s="38"/>
-      <c r="D33" s="38"/>
-      <c r="E33" s="38"/>
-      <c r="F33" s="38"/>
-      <c r="G33" s="38"/>
+      <c r="A33" s="36"/>
+      <c r="B33" s="36"/>
+      <c r="C33" s="36"/>
+      <c r="D33" s="36"/>
+      <c r="E33" s="36"/>
+      <c r="F33" s="36"/>
+      <c r="G33" s="36"/>
     </row>
     <row r="34" spans="1:7" ht="210" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="38"/>
-      <c r="B34" s="38"/>
-      <c r="C34" s="38"/>
-      <c r="D34" s="38"/>
-      <c r="E34" s="38"/>
-      <c r="F34" s="38"/>
-      <c r="G34" s="38"/>
+      <c r="A34" s="36"/>
+      <c r="B34" s="36"/>
+      <c r="C34" s="36"/>
+      <c r="D34" s="36"/>
+      <c r="E34" s="36"/>
+      <c r="F34" s="36"/>
+      <c r="G34" s="36"/>
     </row>
     <row r="35" spans="1:7" ht="135" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="38"/>
-      <c r="B35" s="38"/>
-      <c r="C35" s="38"/>
-      <c r="D35" s="38"/>
-      <c r="E35" s="38"/>
-      <c r="F35" s="38"/>
-      <c r="G35" s="38"/>
+      <c r="A35" s="36"/>
+      <c r="B35" s="36"/>
+      <c r="C35" s="36"/>
+      <c r="D35" s="36"/>
+      <c r="E35" s="36"/>
+      <c r="F35" s="36"/>
+      <c r="G35" s="36"/>
     </row>
     <row r="36" spans="1:7" ht="135" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="38"/>
-      <c r="B36" s="38"/>
-      <c r="C36" s="38"/>
-      <c r="D36" s="38"/>
-      <c r="E36" s="38"/>
-      <c r="F36" s="38"/>
-      <c r="G36" s="38"/>
+      <c r="A36" s="36"/>
+      <c r="B36" s="36"/>
+      <c r="C36" s="36"/>
+      <c r="D36" s="36"/>
+      <c r="E36" s="36"/>
+      <c r="F36" s="36"/>
+      <c r="G36" s="36"/>
     </row>
     <row r="37" spans="1:7" ht="135" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="38"/>
-      <c r="B37" s="38"/>
-      <c r="C37" s="38"/>
-      <c r="D37" s="38"/>
-      <c r="E37" s="38"/>
-      <c r="F37" s="38"/>
-      <c r="G37" s="38"/>
+      <c r="A37" s="36"/>
+      <c r="B37" s="36"/>
+      <c r="C37" s="36"/>
+      <c r="D37" s="36"/>
+      <c r="E37" s="36"/>
+      <c r="F37" s="36"/>
+      <c r="G37" s="36"/>
     </row>
     <row r="38" spans="1:7" ht="135" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="38"/>
-      <c r="B38" s="38"/>
-      <c r="C38" s="38"/>
-      <c r="D38" s="38"/>
-      <c r="E38" s="38"/>
-      <c r="F38" s="38"/>
-      <c r="G38" s="38"/>
+      <c r="A38" s="36"/>
+      <c r="B38" s="36"/>
+      <c r="C38" s="36"/>
+      <c r="D38" s="36"/>
+      <c r="E38" s="36"/>
+      <c r="F38" s="36"/>
+      <c r="G38" s="36"/>
     </row>
     <row r="39" spans="1:7" ht="180" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="38"/>
-      <c r="B39" s="38"/>
-      <c r="C39" s="38"/>
-      <c r="D39" s="38"/>
-      <c r="E39" s="38"/>
-      <c r="F39" s="38"/>
-      <c r="G39" s="38"/>
+      <c r="A39" s="36"/>
+      <c r="B39" s="36"/>
+      <c r="C39" s="36"/>
+      <c r="D39" s="36"/>
+      <c r="E39" s="36"/>
+      <c r="F39" s="36"/>
+      <c r="G39" s="36"/>
     </row>
     <row r="40" spans="1:7" ht="135" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="38"/>
-      <c r="B40" s="38"/>
-      <c r="C40" s="38"/>
-      <c r="D40" s="38"/>
-      <c r="E40" s="38"/>
-      <c r="F40" s="38"/>
-      <c r="G40" s="38"/>
+      <c r="A40" s="36"/>
+      <c r="B40" s="36"/>
+      <c r="C40" s="36"/>
+      <c r="D40" s="36"/>
+      <c r="E40" s="36"/>
+      <c r="F40" s="36"/>
+      <c r="G40" s="36"/>
     </row>
     <row r="41" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="38"/>
-      <c r="B41" s="38"/>
-      <c r="C41" s="38"/>
-      <c r="D41" s="38"/>
-      <c r="E41" s="38"/>
-      <c r="F41" s="38"/>
-      <c r="G41" s="38"/>
+      <c r="A41" s="36"/>
+      <c r="B41" s="36"/>
+      <c r="C41" s="36"/>
+      <c r="D41" s="36"/>
+      <c r="E41" s="36"/>
+      <c r="F41" s="36"/>
+      <c r="G41" s="36"/>
     </row>
     <row r="42" spans="1:7" ht="135" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="38"/>
-      <c r="B42" s="38"/>
-      <c r="C42" s="38"/>
-      <c r="D42" s="38"/>
-      <c r="E42" s="38"/>
-      <c r="F42" s="38"/>
-      <c r="G42" s="38"/>
+      <c r="A42" s="36"/>
+      <c r="B42" s="36"/>
+      <c r="C42" s="36"/>
+      <c r="D42" s="36"/>
+      <c r="E42" s="36"/>
+      <c r="F42" s="36"/>
+      <c r="G42" s="36"/>
     </row>
     <row r="43" spans="1:7" ht="150" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="38"/>
-      <c r="B43" s="38"/>
-      <c r="C43" s="38"/>
-      <c r="D43" s="38"/>
-      <c r="E43" s="38"/>
-      <c r="F43" s="38"/>
-      <c r="G43" s="38"/>
+      <c r="A43" s="36"/>
+      <c r="B43" s="36"/>
+      <c r="C43" s="36"/>
+      <c r="D43" s="36"/>
+      <c r="E43" s="36"/>
+      <c r="F43" s="36"/>
+      <c r="G43" s="36"/>
     </row>
     <row r="44" spans="1:7" ht="150" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="38"/>
-      <c r="B44" s="38"/>
-      <c r="C44" s="38"/>
-      <c r="D44" s="38"/>
-      <c r="E44" s="38"/>
-      <c r="F44" s="38"/>
-      <c r="G44" s="38"/>
+      <c r="A44" s="36"/>
+      <c r="B44" s="36"/>
+      <c r="C44" s="36"/>
+      <c r="D44" s="36"/>
+      <c r="E44" s="36"/>
+      <c r="F44" s="36"/>
+      <c r="G44" s="36"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="38"/>
-      <c r="B45" s="38"/>
-      <c r="C45" s="38"/>
-      <c r="D45" s="38"/>
-      <c r="E45" s="38"/>
-      <c r="F45" s="38"/>
-      <c r="G45" s="38"/>
+      <c r="A45" s="36"/>
+      <c r="B45" s="36"/>
+      <c r="C45" s="36"/>
+      <c r="D45" s="36"/>
+      <c r="E45" s="36"/>
+      <c r="F45" s="36"/>
+      <c r="G45" s="36"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="38"/>
-      <c r="B46" s="38"/>
-      <c r="C46" s="38"/>
-      <c r="D46" s="38"/>
-      <c r="E46" s="38"/>
-      <c r="F46" s="38"/>
-      <c r="G46" s="38"/>
+      <c r="A46" s="36"/>
+      <c r="B46" s="36"/>
+      <c r="C46" s="36"/>
+      <c r="D46" s="36"/>
+      <c r="E46" s="36"/>
+      <c r="F46" s="36"/>
+      <c r="G46" s="36"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="38"/>
-      <c r="B47" s="38"/>
-      <c r="C47" s="38"/>
-      <c r="D47" s="38"/>
-      <c r="E47" s="38"/>
-      <c r="F47" s="38"/>
-      <c r="G47" s="38"/>
+      <c r="A47" s="36"/>
+      <c r="B47" s="36"/>
+      <c r="C47" s="36"/>
+      <c r="D47" s="36"/>
+      <c r="E47" s="36"/>
+      <c r="F47" s="36"/>
+      <c r="G47" s="36"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="38"/>
-      <c r="B48" s="38"/>
-      <c r="C48" s="38"/>
-      <c r="D48" s="38"/>
-      <c r="E48" s="38"/>
-      <c r="F48" s="38"/>
-      <c r="G48" s="38"/>
+      <c r="A48" s="36"/>
+      <c r="B48" s="36"/>
+      <c r="C48" s="36"/>
+      <c r="D48" s="36"/>
+      <c r="E48" s="36"/>
+      <c r="F48" s="36"/>
+      <c r="G48" s="36"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="38"/>
-      <c r="B49" s="38"/>
-      <c r="C49" s="38"/>
-      <c r="D49" s="38"/>
-      <c r="E49" s="38"/>
-      <c r="F49" s="38"/>
-      <c r="G49" s="38"/>
+      <c r="A49" s="36"/>
+      <c r="B49" s="36"/>
+      <c r="C49" s="36"/>
+      <c r="D49" s="36"/>
+      <c r="E49" s="36"/>
+      <c r="F49" s="36"/>
+      <c r="G49" s="36"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="38"/>
-      <c r="B50" s="38"/>
-      <c r="C50" s="38"/>
-      <c r="D50" s="38"/>
-      <c r="E50" s="38"/>
-      <c r="F50" s="38"/>
-      <c r="G50" s="38"/>
+      <c r="A50" s="36"/>
+      <c r="B50" s="36"/>
+      <c r="C50" s="36"/>
+      <c r="D50" s="36"/>
+      <c r="E50" s="36"/>
+      <c r="F50" s="36"/>
+      <c r="G50" s="36"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="38"/>
-      <c r="B51" s="38"/>
-      <c r="C51" s="38"/>
-      <c r="D51" s="38"/>
-      <c r="E51" s="38"/>
-      <c r="F51" s="38"/>
-      <c r="G51" s="38"/>
+      <c r="A51" s="36"/>
+      <c r="B51" s="36"/>
+      <c r="C51" s="36"/>
+      <c r="D51" s="36"/>
+      <c r="E51" s="36"/>
+      <c r="F51" s="36"/>
+      <c r="G51" s="36"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="38"/>
-      <c r="B52" s="38"/>
-      <c r="C52" s="38"/>
-      <c r="D52" s="38"/>
-      <c r="E52" s="38"/>
-      <c r="F52" s="38"/>
-      <c r="G52" s="38"/>
+      <c r="A52" s="36"/>
+      <c r="B52" s="36"/>
+      <c r="C52" s="36"/>
+      <c r="D52" s="36"/>
+      <c r="E52" s="36"/>
+      <c r="F52" s="36"/>
+      <c r="G52" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>